<commit_message>
Publish LeeValley_2015_WCH, Pau_2015_WC, Prague_2013_WCH
</commit_message>
<xml_diff>
--- a/events/LeeValley_2015_WCH/LeeValley_2015_WCH_start.xlsx
+++ b/events/LeeValley_2015_WCH/LeeValley_2015_WCH_start.xlsx
@@ -13374,7 +13374,7 @@
       </c>
       <c r="I218" t="inlineStr">
         <is>
-          <t>LIB</t>
+          <t>LBN</t>
         </is>
       </c>
       <c r="J218" t="n">
@@ -19934,7 +19934,7 @@
       </c>
       <c r="I333" t="inlineStr">
         <is>
-          <t>LIB</t>
+          <t>LBN</t>
         </is>
       </c>
       <c r="J333" t="n">

</xml_diff>

<commit_message>
Publish LaSeu_2016_WC, LeeValley_2015_WCH, Pau_2015_WC, Prague_2013_WCH
</commit_message>
<xml_diff>
--- a/events/LeeValley_2015_WCH/LeeValley_2015_WCH_start.xlsx
+++ b/events/LeeValley_2015_WCH/LeeValley_2015_WCH_start.xlsx
@@ -13388,6 +13388,11 @@
           <t>MERJAN Richard</t>
         </is>
       </c>
+      <c r="X218" t="inlineStr">
+        <is>
+          <t>45918</t>
+        </is>
+      </c>
     </row>
     <row r="219">
       <c r="A219" t="inlineStr">
@@ -19946,6 +19951,11 @@
       <c r="R333" t="inlineStr">
         <is>
           <t>MERJAN Richard</t>
+        </is>
+      </c>
+      <c r="X333" t="inlineStr">
+        <is>
+          <t>45918</t>
         </is>
       </c>
     </row>

</xml_diff>